<commit_message>
MIA: run automatico 2026-07-28 14:07 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F141"/>
+  <dimension ref="A1:F142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3232,19 +3232,39 @@
         <v>46230</v>
       </c>
       <c r="B141" t="n">
-        <v>3.22</v>
+        <v>3.220000028610229</v>
       </c>
       <c r="C141" t="n">
-        <v>3.27</v>
+        <v>3.269999980926514</v>
       </c>
       <c r="D141" t="n">
-        <v>3.21</v>
+        <v>3.210000038146973</v>
       </c>
       <c r="E141" t="n">
-        <v>3.27</v>
+        <v>3.269999980926514</v>
       </c>
       <c r="F141" t="n">
         <v>1750700</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B142" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="C142" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="D142" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="E142" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F142" t="n">
+        <v>411400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-07-28 18:21 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -3252,10 +3252,10 @@
         <v>46231</v>
       </c>
       <c r="B142" t="n">
-        <v>3.29</v>
+        <v>3.35</v>
       </c>
       <c r="C142" t="n">
-        <v>3.31</v>
+        <v>3.36</v>
       </c>
       <c r="D142" t="n">
         <v>3.27</v>
@@ -3264,7 +3264,7 @@
         <v>3.27</v>
       </c>
       <c r="F142" t="n">
-        <v>411400</v>
+        <v>1915700</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-07-28 21:44 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -3252,7 +3252,7 @@
         <v>46231</v>
       </c>
       <c r="B142" t="n">
-        <v>3.35</v>
+        <v>3.29</v>
       </c>
       <c r="C142" t="n">
         <v>3.36</v>
@@ -3264,7 +3264,7 @@
         <v>3.27</v>
       </c>
       <c r="F142" t="n">
-        <v>1915700</v>
+        <v>2817100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-07-29 12:04 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -3252,16 +3252,16 @@
         <v>46231</v>
       </c>
       <c r="B142" t="n">
-        <v>3.29</v>
+        <v>3.289999961853027</v>
       </c>
       <c r="C142" t="n">
-        <v>3.36</v>
+        <v>3.359999895095825</v>
       </c>
       <c r="D142" t="n">
-        <v>3.27</v>
+        <v>3.269999980926514</v>
       </c>
       <c r="E142" t="n">
-        <v>3.27</v>
+        <v>3.269999980926514</v>
       </c>
       <c r="F142" t="n">
         <v>2817100</v>

</xml_diff>

<commit_message>
MIA: run automatico 2026-07-29 21:32 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -3272,10 +3272,10 @@
         <v>46232</v>
       </c>
       <c r="B143" t="n">
-        <v>3.34</v>
+        <v>3.35</v>
       </c>
       <c r="C143" t="n">
-        <v>3.37</v>
+        <v>3.38</v>
       </c>
       <c r="D143" t="n">
         <v>3.25</v>
@@ -3284,7 +3284,7 @@
         <v>3.26</v>
       </c>
       <c r="F143" t="n">
-        <v>1939000</v>
+        <v>2720100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-07-30 22:45 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F143"/>
+  <dimension ref="A1:F144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3272,19 +3272,39 @@
         <v>46232</v>
       </c>
       <c r="B143" t="n">
-        <v>3.35</v>
+        <v>3.349999904632568</v>
       </c>
       <c r="C143" t="n">
-        <v>3.38</v>
+        <v>3.380000114440918</v>
       </c>
       <c r="D143" t="n">
         <v>3.25</v>
       </c>
       <c r="E143" t="n">
-        <v>3.26</v>
+        <v>3.259999990463257</v>
       </c>
       <c r="F143" t="n">
         <v>2720100</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="1" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B144" t="n">
+        <v>3.39</v>
+      </c>
+      <c r="C144" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="D144" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="E144" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="F144" t="n">
+        <v>2171100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-07-31 22:41 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F144"/>
+  <dimension ref="A1:F145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3292,19 +3292,39 @@
         <v>46233</v>
       </c>
       <c r="B144" t="n">
-        <v>3.39</v>
+        <v>3.390000104904175</v>
       </c>
       <c r="C144" t="n">
-        <v>3.42</v>
+        <v>3.420000076293945</v>
       </c>
       <c r="D144" t="n">
-        <v>3.31</v>
+        <v>3.309999942779541</v>
       </c>
       <c r="E144" t="n">
-        <v>3.31</v>
+        <v>3.309999942779541</v>
       </c>
       <c r="F144" t="n">
         <v>2171100</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B145" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="C145" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="D145" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="E145" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="F145" t="n">
+        <v>2644500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-03 22:40 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F145"/>
+  <dimension ref="A1:F146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3312,19 +3312,39 @@
         <v>46234</v>
       </c>
       <c r="B145" t="n">
+        <v>3.490000009536743</v>
+      </c>
+      <c r="C145" t="n">
+        <v>3.539999961853027</v>
+      </c>
+      <c r="D145" t="n">
+        <v>3.380000114440918</v>
+      </c>
+      <c r="E145" t="n">
+        <v>3.380000114440918</v>
+      </c>
+      <c r="F145" t="n">
+        <v>2644700</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B146" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="C146" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="D146" t="n">
         <v>3.49</v>
       </c>
-      <c r="C145" t="n">
-        <v>3.54</v>
-      </c>
-      <c r="D145" t="n">
-        <v>3.38</v>
-      </c>
-      <c r="E145" t="n">
-        <v>3.38</v>
-      </c>
-      <c r="F145" t="n">
-        <v>2644500</v>
+      <c r="E146" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F146" t="n">
+        <v>6262900</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-04 22:45 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -3309,42 +3309,42 @@
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="B145" t="n">
+        <v>3.650000095367432</v>
+      </c>
+      <c r="C145" t="n">
+        <v>3.670000076293945</v>
+      </c>
+      <c r="D145" t="n">
         <v>3.490000009536743</v>
       </c>
-      <c r="C145" t="n">
-        <v>3.539999961853027</v>
-      </c>
-      <c r="D145" t="n">
-        <v>3.380000114440918</v>
-      </c>
       <c r="E145" t="n">
-        <v>3.380000114440918</v>
+        <v>3.5</v>
       </c>
       <c r="F145" t="n">
-        <v>2644700</v>
+        <v>6262900</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B146" t="n">
-        <v>3.65</v>
+        <v>3.68</v>
       </c>
       <c r="C146" t="n">
-        <v>3.67</v>
+        <v>3.78</v>
       </c>
       <c r="D146" t="n">
-        <v>3.49</v>
+        <v>3.59</v>
       </c>
       <c r="E146" t="n">
-        <v>3.5</v>
+        <v>3.66</v>
       </c>
       <c r="F146" t="n">
-        <v>6262900</v>
+        <v>5049200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-05 22:42 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F146"/>
+  <dimension ref="A1:F148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3309,42 +3309,82 @@
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
-        <v>46237</v>
+        <v>46234</v>
       </c>
       <c r="B145" t="n">
-        <v>3.650000095367432</v>
+        <v>3.490000009536743</v>
       </c>
       <c r="C145" t="n">
-        <v>3.670000076293945</v>
+        <v>3.539999961853027</v>
       </c>
       <c r="D145" t="n">
-        <v>3.490000009536743</v>
+        <v>3.380000114440918</v>
       </c>
       <c r="E145" t="n">
-        <v>3.5</v>
+        <v>3.380000114440918</v>
       </c>
       <c r="F145" t="n">
-        <v>6262900</v>
+        <v>2644700</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B146" t="n">
+        <v>3.650000095367432</v>
+      </c>
+      <c r="C146" t="n">
+        <v>3.670000076293945</v>
+      </c>
+      <c r="D146" t="n">
+        <v>3.490000009536743</v>
+      </c>
+      <c r="E146" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F146" t="n">
+        <v>6262900</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="1" t="n">
         <v>46238</v>
       </c>
-      <c r="B146" t="n">
-        <v>3.68</v>
-      </c>
-      <c r="C146" t="n">
-        <v>3.78</v>
-      </c>
-      <c r="D146" t="n">
-        <v>3.59</v>
-      </c>
-      <c r="E146" t="n">
-        <v>3.66</v>
-      </c>
-      <c r="F146" t="n">
+      <c r="B147" t="n">
+        <v>3.680000066757202</v>
+      </c>
+      <c r="C147" t="n">
+        <v>3.779999971389771</v>
+      </c>
+      <c r="D147" t="n">
+        <v>3.589999914169312</v>
+      </c>
+      <c r="E147" t="n">
+        <v>3.660000085830688</v>
+      </c>
+      <c r="F147" t="n">
         <v>5049200</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="1" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B148" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="C148" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="D148" t="n">
+        <v>3.61</v>
+      </c>
+      <c r="E148" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="F148" t="n">
+        <v>1946500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-06 23:18 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F148"/>
+  <dimension ref="A1:F149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3372,19 +3372,39 @@
         <v>46239</v>
       </c>
       <c r="B148" t="n">
-        <v>3.62</v>
+        <v>3.619999885559082</v>
       </c>
       <c r="C148" t="n">
-        <v>3.71</v>
+        <v>3.710000038146973</v>
       </c>
       <c r="D148" t="n">
-        <v>3.61</v>
+        <v>3.609999895095825</v>
       </c>
       <c r="E148" t="n">
-        <v>3.71</v>
+        <v>3.710000038146973</v>
       </c>
       <c r="F148" t="n">
         <v>1946500</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="B149" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="C149" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="D149" t="n">
+        <v>3.52</v>
+      </c>
+      <c r="E149" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="F149" t="n">
+        <v>2415500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-07 22:14 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -3309,102 +3309,102 @@
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="B145" t="n">
+        <v>3.650000095367432</v>
+      </c>
+      <c r="C145" t="n">
+        <v>3.670000076293945</v>
+      </c>
+      <c r="D145" t="n">
         <v>3.490000009536743</v>
       </c>
-      <c r="C145" t="n">
-        <v>3.539999961853027</v>
-      </c>
-      <c r="D145" t="n">
-        <v>3.380000114440918</v>
-      </c>
       <c r="E145" t="n">
-        <v>3.380000114440918</v>
+        <v>3.5</v>
       </c>
       <c r="F145" t="n">
-        <v>2644700</v>
+        <v>6262900</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B146" t="n">
-        <v>3.650000095367432</v>
+        <v>3.680000066757202</v>
       </c>
       <c r="C146" t="n">
-        <v>3.670000076293945</v>
+        <v>3.779999971389771</v>
       </c>
       <c r="D146" t="n">
-        <v>3.490000009536743</v>
+        <v>3.589999914169312</v>
       </c>
       <c r="E146" t="n">
-        <v>3.5</v>
+        <v>3.660000085830688</v>
       </c>
       <c r="F146" t="n">
-        <v>6262900</v>
+        <v>5049200</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="B147" t="n">
-        <v>3.680000066757202</v>
+        <v>3.619999885559082</v>
       </c>
       <c r="C147" t="n">
-        <v>3.779999971389771</v>
+        <v>3.710000038146973</v>
       </c>
       <c r="D147" t="n">
-        <v>3.589999914169312</v>
+        <v>3.609999895095825</v>
       </c>
       <c r="E147" t="n">
-        <v>3.660000085830688</v>
+        <v>3.710000038146973</v>
       </c>
       <c r="F147" t="n">
-        <v>5049200</v>
+        <v>1946500</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="B148" t="n">
+        <v>3.569999933242798</v>
+      </c>
+      <c r="C148" t="n">
         <v>3.619999885559082</v>
       </c>
-      <c r="C148" t="n">
-        <v>3.710000038146973</v>
-      </c>
       <c r="D148" t="n">
-        <v>3.609999895095825</v>
+        <v>3.519999980926514</v>
       </c>
       <c r="E148" t="n">
-        <v>3.710000038146973</v>
+        <v>3.569999933242798</v>
       </c>
       <c r="F148" t="n">
-        <v>1946500</v>
+        <v>2415500</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="B149" t="n">
-        <v>3.57</v>
+        <v>3.52</v>
       </c>
       <c r="C149" t="n">
-        <v>3.62</v>
+        <v>3.6</v>
       </c>
       <c r="D149" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="E149" t="n">
         <v>3.52</v>
       </c>
-      <c r="E149" t="n">
-        <v>3.57</v>
-      </c>
       <c r="F149" t="n">
-        <v>2415500</v>
+        <v>2618900</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-10 22:15 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F149"/>
+  <dimension ref="A1:F151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3309,102 +3309,142 @@
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
-        <v>46237</v>
+        <v>46234</v>
       </c>
       <c r="B145" t="n">
-        <v>3.650000095367432</v>
+        <v>3.490000009536743</v>
       </c>
       <c r="C145" t="n">
-        <v>3.670000076293945</v>
+        <v>3.539999961853027</v>
       </c>
       <c r="D145" t="n">
-        <v>3.490000009536743</v>
+        <v>3.380000114440918</v>
       </c>
       <c r="E145" t="n">
-        <v>3.5</v>
+        <v>3.380000114440918</v>
       </c>
       <c r="F145" t="n">
-        <v>6262900</v>
+        <v>2644700</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
-        <v>46238</v>
+        <v>46237</v>
       </c>
       <c r="B146" t="n">
-        <v>3.680000066757202</v>
+        <v>3.650000095367432</v>
       </c>
       <c r="C146" t="n">
-        <v>3.779999971389771</v>
+        <v>3.670000076293945</v>
       </c>
       <c r="D146" t="n">
-        <v>3.589999914169312</v>
+        <v>3.490000009536743</v>
       </c>
       <c r="E146" t="n">
-        <v>3.660000085830688</v>
+        <v>3.5</v>
       </c>
       <c r="F146" t="n">
-        <v>5049200</v>
+        <v>6262900</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
-        <v>46239</v>
+        <v>46238</v>
       </c>
       <c r="B147" t="n">
-        <v>3.619999885559082</v>
+        <v>3.680000066757202</v>
       </c>
       <c r="C147" t="n">
-        <v>3.710000038146973</v>
+        <v>3.779999971389771</v>
       </c>
       <c r="D147" t="n">
-        <v>3.609999895095825</v>
+        <v>3.589999914169312</v>
       </c>
       <c r="E147" t="n">
-        <v>3.710000038146973</v>
+        <v>3.660000085830688</v>
       </c>
       <c r="F147" t="n">
-        <v>1946500</v>
+        <v>5049200</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
-        <v>46240</v>
+        <v>46239</v>
       </c>
       <c r="B148" t="n">
-        <v>3.569999933242798</v>
+        <v>3.619999885559082</v>
       </c>
       <c r="C148" t="n">
-        <v>3.619999885559082</v>
+        <v>3.710000038146973</v>
       </c>
       <c r="D148" t="n">
-        <v>3.519999980926514</v>
+        <v>3.609999895095825</v>
       </c>
       <c r="E148" t="n">
-        <v>3.569999933242798</v>
+        <v>3.710000038146973</v>
       </c>
       <c r="F148" t="n">
-        <v>2415500</v>
+        <v>1946500</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="B149" t="n">
+        <v>3.569999933242798</v>
+      </c>
+      <c r="C149" t="n">
+        <v>3.619999885559082</v>
+      </c>
+      <c r="D149" t="n">
+        <v>3.519999980926514</v>
+      </c>
+      <c r="E149" t="n">
+        <v>3.569999933242798</v>
+      </c>
+      <c r="F149" t="n">
+        <v>2415500</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="1" t="n">
         <v>46241</v>
       </c>
-      <c r="B149" t="n">
-        <v>3.52</v>
-      </c>
-      <c r="C149" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="D149" t="n">
-        <v>3.44</v>
-      </c>
-      <c r="E149" t="n">
-        <v>3.52</v>
-      </c>
-      <c r="F149" t="n">
+      <c r="B150" t="n">
+        <v>3.519999980926514</v>
+      </c>
+      <c r="C150" t="n">
+        <v>3.599999904632568</v>
+      </c>
+      <c r="D150" t="n">
+        <v>3.440000057220459</v>
+      </c>
+      <c r="E150" t="n">
+        <v>3.519999980926514</v>
+      </c>
+      <c r="F150" t="n">
         <v>2618900</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B151" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="C151" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D151" t="n">
+        <v>3.39</v>
+      </c>
+      <c r="E151" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F151" t="n">
+        <v>2613600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-11 22:26 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F151"/>
+  <dimension ref="A1:F152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3432,19 +3432,39 @@
         <v>46244</v>
       </c>
       <c r="B151" t="n">
-        <v>3.41</v>
+        <v>3.410000085830688</v>
       </c>
       <c r="C151" t="n">
         <v>3.5</v>
       </c>
       <c r="D151" t="n">
-        <v>3.39</v>
+        <v>3.390000104904175</v>
       </c>
       <c r="E151" t="n">
-        <v>3.45</v>
+        <v>3.450000047683716</v>
       </c>
       <c r="F151" t="n">
         <v>2613600</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="1" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B152" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="C152" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="D152" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="E152" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="F152" t="n">
+        <v>5077500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-13 22:26 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F152"/>
+  <dimension ref="A1:F153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3452,19 +3452,39 @@
         <v>46246</v>
       </c>
       <c r="B152" t="n">
-        <v>3.36</v>
+        <v>3.359999895095825</v>
       </c>
       <c r="C152" t="n">
-        <v>3.4</v>
+        <v>3.400000095367432</v>
       </c>
       <c r="D152" t="n">
-        <v>3.28</v>
+        <v>3.279999971389771</v>
       </c>
       <c r="E152" t="n">
-        <v>3.34</v>
+        <v>3.339999914169312</v>
       </c>
       <c r="F152" t="n">
         <v>4336100</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="1" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B153" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="C153" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="D153" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="E153" t="n">
+        <v>3.39</v>
+      </c>
+      <c r="F153" t="n">
+        <v>3777900</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-14 21:58 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -3129,90 +3129,90 @@
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B136" t="n">
-        <v>3.160000085830688</v>
+        <v>3.140000104904175</v>
       </c>
       <c r="C136" t="n">
-        <v>3.200000047683716</v>
+        <v>3.170000076293945</v>
       </c>
       <c r="D136" t="n">
-        <v>3.079999923706055</v>
+        <v>3.089999914169312</v>
       </c>
       <c r="E136" t="n">
-        <v>3.079999923706055</v>
+        <v>3.130000114440918</v>
       </c>
       <c r="F136" t="n">
-        <v>2046300</v>
+        <v>2828500</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="B137" t="n">
-        <v>3.140000104904175</v>
+        <v>3.230000019073486</v>
       </c>
       <c r="C137" t="n">
-        <v>3.170000076293945</v>
+        <v>3.259999990463257</v>
       </c>
       <c r="D137" t="n">
-        <v>3.089999914169312</v>
+        <v>3.099999904632568</v>
       </c>
       <c r="E137" t="n">
         <v>3.130000114440918</v>
       </c>
       <c r="F137" t="n">
-        <v>2828500</v>
+        <v>3830200</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="B138" t="n">
-        <v>3.230000019073486</v>
+        <v>3.279999971389771</v>
       </c>
       <c r="C138" t="n">
-        <v>3.259999990463257</v>
+        <v>3.329999923706055</v>
       </c>
       <c r="D138" t="n">
-        <v>3.099999904632568</v>
+        <v>3.190000057220459</v>
       </c>
       <c r="E138" t="n">
-        <v>3.130000114440918</v>
+        <v>3.190000057220459</v>
       </c>
       <c r="F138" t="n">
-        <v>3830200</v>
+        <v>3736000</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="B139" t="n">
-        <v>3.279999971389771</v>
+        <v>3.259999990463257</v>
       </c>
       <c r="C139" t="n">
-        <v>3.329999923706055</v>
+        <v>3.269999980926514</v>
       </c>
       <c r="D139" t="n">
-        <v>3.190000057220459</v>
+        <v>3.210000038146973</v>
       </c>
       <c r="E139" t="n">
-        <v>3.190000057220459</v>
+        <v>3.259999990463257</v>
       </c>
       <c r="F139" t="n">
-        <v>3736000</v>
+        <v>1448700</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="B140" t="n">
-        <v>3.259999990463257</v>
+        <v>3.220000028610229</v>
       </c>
       <c r="C140" t="n">
         <v>3.269999980926514</v>
@@ -3221,270 +3221,270 @@
         <v>3.210000038146973</v>
       </c>
       <c r="E140" t="n">
-        <v>3.259999990463257</v>
+        <v>3.269999980926514</v>
       </c>
       <c r="F140" t="n">
-        <v>1448700</v>
+        <v>1750700</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B141" t="n">
-        <v>3.220000028610229</v>
+        <v>3.289999961853027</v>
       </c>
       <c r="C141" t="n">
+        <v>3.359999895095825</v>
+      </c>
+      <c r="D141" t="n">
         <v>3.269999980926514</v>
-      </c>
-      <c r="D141" t="n">
-        <v>3.210000038146973</v>
       </c>
       <c r="E141" t="n">
         <v>3.269999980926514</v>
       </c>
       <c r="F141" t="n">
-        <v>1750700</v>
+        <v>2817100</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B142" t="n">
-        <v>3.289999961853027</v>
+        <v>3.349999904632568</v>
       </c>
       <c r="C142" t="n">
-        <v>3.359999895095825</v>
+        <v>3.380000114440918</v>
       </c>
       <c r="D142" t="n">
-        <v>3.269999980926514</v>
+        <v>3.25</v>
       </c>
       <c r="E142" t="n">
-        <v>3.269999980926514</v>
+        <v>3.259999990463257</v>
       </c>
       <c r="F142" t="n">
-        <v>2817100</v>
+        <v>2720100</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B143" t="n">
-        <v>3.349999904632568</v>
+        <v>3.390000104904175</v>
       </c>
       <c r="C143" t="n">
-        <v>3.380000114440918</v>
+        <v>3.420000076293945</v>
       </c>
       <c r="D143" t="n">
-        <v>3.25</v>
+        <v>3.309999942779541</v>
       </c>
       <c r="E143" t="n">
-        <v>3.259999990463257</v>
+        <v>3.309999942779541</v>
       </c>
       <c r="F143" t="n">
-        <v>2720100</v>
+        <v>2171100</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
-        <v>46233</v>
+        <v>46237</v>
       </c>
       <c r="B144" t="n">
-        <v>3.390000104904175</v>
+        <v>3.650000095367432</v>
       </c>
       <c r="C144" t="n">
-        <v>3.420000076293945</v>
+        <v>3.670000076293945</v>
       </c>
       <c r="D144" t="n">
-        <v>3.309999942779541</v>
+        <v>3.490000009536743</v>
       </c>
       <c r="E144" t="n">
-        <v>3.309999942779541</v>
+        <v>3.5</v>
       </c>
       <c r="F144" t="n">
-        <v>2171100</v>
+        <v>6262900</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B145" t="n">
-        <v>3.650000095367432</v>
+        <v>3.680000066757202</v>
       </c>
       <c r="C145" t="n">
-        <v>3.670000076293945</v>
+        <v>3.779999971389771</v>
       </c>
       <c r="D145" t="n">
-        <v>3.490000009536743</v>
+        <v>3.589999914169312</v>
       </c>
       <c r="E145" t="n">
-        <v>3.5</v>
+        <v>3.660000085830688</v>
       </c>
       <c r="F145" t="n">
-        <v>6262900</v>
+        <v>5049200</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="B146" t="n">
-        <v>3.680000066757202</v>
+        <v>3.619999885559082</v>
       </c>
       <c r="C146" t="n">
-        <v>3.779999971389771</v>
+        <v>3.710000038146973</v>
       </c>
       <c r="D146" t="n">
-        <v>3.589999914169312</v>
+        <v>3.609999895095825</v>
       </c>
       <c r="E146" t="n">
-        <v>3.660000085830688</v>
+        <v>3.710000038146973</v>
       </c>
       <c r="F146" t="n">
-        <v>5049200</v>
+        <v>1946500</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="B147" t="n">
+        <v>3.569999933242798</v>
+      </c>
+      <c r="C147" t="n">
         <v>3.619999885559082</v>
       </c>
-      <c r="C147" t="n">
-        <v>3.710000038146973</v>
-      </c>
       <c r="D147" t="n">
-        <v>3.609999895095825</v>
+        <v>3.519999980926514</v>
       </c>
       <c r="E147" t="n">
-        <v>3.710000038146973</v>
+        <v>3.569999933242798</v>
       </c>
       <c r="F147" t="n">
-        <v>1946500</v>
+        <v>2415500</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="B148" t="n">
-        <v>3.569999933242798</v>
+        <v>3.519999980926514</v>
       </c>
       <c r="C148" t="n">
-        <v>3.619999885559082</v>
+        <v>3.599999904632568</v>
       </c>
       <c r="D148" t="n">
+        <v>3.440000057220459</v>
+      </c>
+      <c r="E148" t="n">
         <v>3.519999980926514</v>
       </c>
-      <c r="E148" t="n">
-        <v>3.569999933242798</v>
-      </c>
       <c r="F148" t="n">
-        <v>2415500</v>
+        <v>2618900</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="B149" t="n">
-        <v>3.519999980926514</v>
+        <v>3.410000085830688</v>
       </c>
       <c r="C149" t="n">
-        <v>3.599999904632568</v>
+        <v>3.5</v>
       </c>
       <c r="D149" t="n">
-        <v>3.440000057220459</v>
+        <v>3.390000104904175</v>
       </c>
       <c r="E149" t="n">
-        <v>3.519999980926514</v>
+        <v>3.450000047683716</v>
       </c>
       <c r="F149" t="n">
-        <v>2618900</v>
+        <v>2613600</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="B150" t="n">
-        <v>3.410000085830688</v>
+        <v>3.319999933242798</v>
       </c>
       <c r="C150" t="n">
-        <v>3.5</v>
+        <v>3.440000057220459</v>
       </c>
       <c r="D150" t="n">
-        <v>3.390000104904175</v>
+        <v>3.309999942779541</v>
       </c>
       <c r="E150" t="n">
-        <v>3.450000047683716</v>
+        <v>3.369999885559082</v>
       </c>
       <c r="F150" t="n">
-        <v>2613600</v>
+        <v>5077500</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="B151" t="n">
-        <v>3.319999933242798</v>
+        <v>3.359999895095825</v>
       </c>
       <c r="C151" t="n">
-        <v>3.440000057220459</v>
+        <v>3.400000095367432</v>
       </c>
       <c r="D151" t="n">
-        <v>3.309999942779541</v>
+        <v>3.279999971389771</v>
       </c>
       <c r="E151" t="n">
-        <v>3.369999885559082</v>
+        <v>3.339999914169312</v>
       </c>
       <c r="F151" t="n">
-        <v>5077500</v>
+        <v>4336100</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="B152" t="n">
-        <v>3.359999895095825</v>
+        <v>3.450000047683716</v>
       </c>
       <c r="C152" t="n">
-        <v>3.400000095367432</v>
+        <v>3.470000028610229</v>
       </c>
       <c r="D152" t="n">
-        <v>3.279999971389771</v>
+        <v>3.369999885559082</v>
       </c>
       <c r="E152" t="n">
-        <v>3.339999914169312</v>
+        <v>3.390000104904175</v>
       </c>
       <c r="F152" t="n">
-        <v>4336100</v>
+        <v>3777900</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="B153" t="n">
-        <v>3.45</v>
+        <v>3.16</v>
       </c>
       <c r="C153" t="n">
-        <v>3.47</v>
+        <v>3.42</v>
       </c>
       <c r="D153" t="n">
-        <v>3.37</v>
+        <v>3.09</v>
       </c>
       <c r="E153" t="n">
-        <v>3.39</v>
+        <v>3.41</v>
       </c>
       <c r="F153" t="n">
-        <v>3777900</v>
+        <v>12069700</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-17 21:58 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F153"/>
+  <dimension ref="A1:F156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3129,90 +3129,90 @@
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
-        <v>46224</v>
+        <v>46223</v>
       </c>
       <c r="B136" t="n">
-        <v>3.140000104904175</v>
+        <v>3.160000085830688</v>
       </c>
       <c r="C136" t="n">
-        <v>3.170000076293945</v>
+        <v>3.200000047683716</v>
       </c>
       <c r="D136" t="n">
-        <v>3.089999914169312</v>
+        <v>3.079999923706055</v>
       </c>
       <c r="E136" t="n">
-        <v>3.130000114440918</v>
+        <v>3.079999923706055</v>
       </c>
       <c r="F136" t="n">
-        <v>2828500</v>
+        <v>2046300</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
-        <v>46225</v>
+        <v>46224</v>
       </c>
       <c r="B137" t="n">
-        <v>3.230000019073486</v>
+        <v>3.140000104904175</v>
       </c>
       <c r="C137" t="n">
-        <v>3.259999990463257</v>
+        <v>3.170000076293945</v>
       </c>
       <c r="D137" t="n">
-        <v>3.099999904632568</v>
+        <v>3.089999914169312</v>
       </c>
       <c r="E137" t="n">
         <v>3.130000114440918</v>
       </c>
       <c r="F137" t="n">
-        <v>3830200</v>
+        <v>2828500</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
-        <v>46226</v>
+        <v>46225</v>
       </c>
       <c r="B138" t="n">
-        <v>3.279999971389771</v>
+        <v>3.230000019073486</v>
       </c>
       <c r="C138" t="n">
-        <v>3.329999923706055</v>
+        <v>3.259999990463257</v>
       </c>
       <c r="D138" t="n">
-        <v>3.190000057220459</v>
+        <v>3.099999904632568</v>
       </c>
       <c r="E138" t="n">
-        <v>3.190000057220459</v>
+        <v>3.130000114440918</v>
       </c>
       <c r="F138" t="n">
-        <v>3736000</v>
+        <v>3830200</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
-        <v>46227</v>
+        <v>46226</v>
       </c>
       <c r="B139" t="n">
-        <v>3.259999990463257</v>
+        <v>3.279999971389771</v>
       </c>
       <c r="C139" t="n">
-        <v>3.269999980926514</v>
+        <v>3.329999923706055</v>
       </c>
       <c r="D139" t="n">
-        <v>3.210000038146973</v>
+        <v>3.190000057220459</v>
       </c>
       <c r="E139" t="n">
-        <v>3.259999990463257</v>
+        <v>3.190000057220459</v>
       </c>
       <c r="F139" t="n">
-        <v>1448700</v>
+        <v>3736000</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
-        <v>46230</v>
+        <v>46227</v>
       </c>
       <c r="B140" t="n">
-        <v>3.220000028610229</v>
+        <v>3.259999990463257</v>
       </c>
       <c r="C140" t="n">
         <v>3.269999980926514</v>
@@ -3221,270 +3221,330 @@
         <v>3.210000038146973</v>
       </c>
       <c r="E140" t="n">
-        <v>3.269999980926514</v>
+        <v>3.259999990463257</v>
       </c>
       <c r="F140" t="n">
-        <v>1750700</v>
+        <v>1448700</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
-        <v>46231</v>
+        <v>46230</v>
       </c>
       <c r="B141" t="n">
-        <v>3.289999961853027</v>
+        <v>3.220000028610229</v>
       </c>
       <c r="C141" t="n">
-        <v>3.359999895095825</v>
+        <v>3.269999980926514</v>
       </c>
       <c r="D141" t="n">
-        <v>3.269999980926514</v>
+        <v>3.210000038146973</v>
       </c>
       <c r="E141" t="n">
         <v>3.269999980926514</v>
       </c>
       <c r="F141" t="n">
-        <v>2817100</v>
+        <v>1750700</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
-        <v>46232</v>
+        <v>46231</v>
       </c>
       <c r="B142" t="n">
-        <v>3.349999904632568</v>
+        <v>3.289999961853027</v>
       </c>
       <c r="C142" t="n">
-        <v>3.380000114440918</v>
+        <v>3.359999895095825</v>
       </c>
       <c r="D142" t="n">
-        <v>3.25</v>
+        <v>3.269999980926514</v>
       </c>
       <c r="E142" t="n">
-        <v>3.259999990463257</v>
+        <v>3.269999980926514</v>
       </c>
       <c r="F142" t="n">
-        <v>2720100</v>
+        <v>2817100</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
-        <v>46233</v>
+        <v>46232</v>
       </c>
       <c r="B143" t="n">
-        <v>3.390000104904175</v>
+        <v>3.349999904632568</v>
       </c>
       <c r="C143" t="n">
-        <v>3.420000076293945</v>
+        <v>3.380000114440918</v>
       </c>
       <c r="D143" t="n">
-        <v>3.309999942779541</v>
+        <v>3.25</v>
       </c>
       <c r="E143" t="n">
-        <v>3.309999942779541</v>
+        <v>3.259999990463257</v>
       </c>
       <c r="F143" t="n">
-        <v>2171100</v>
+        <v>2720100</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
-        <v>46237</v>
+        <v>46233</v>
       </c>
       <c r="B144" t="n">
-        <v>3.650000095367432</v>
+        <v>3.390000104904175</v>
       </c>
       <c r="C144" t="n">
-        <v>3.670000076293945</v>
+        <v>3.420000076293945</v>
       </c>
       <c r="D144" t="n">
-        <v>3.490000009536743</v>
+        <v>3.309999942779541</v>
       </c>
       <c r="E144" t="n">
-        <v>3.5</v>
+        <v>3.309999942779541</v>
       </c>
       <c r="F144" t="n">
-        <v>6262900</v>
+        <v>2171100</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
-        <v>46238</v>
+        <v>46234</v>
       </c>
       <c r="B145" t="n">
-        <v>3.680000066757202</v>
+        <v>3.490000009536743</v>
       </c>
       <c r="C145" t="n">
-        <v>3.779999971389771</v>
+        <v>3.539999961853027</v>
       </c>
       <c r="D145" t="n">
-        <v>3.589999914169312</v>
+        <v>3.380000114440918</v>
       </c>
       <c r="E145" t="n">
-        <v>3.660000085830688</v>
+        <v>3.380000114440918</v>
       </c>
       <c r="F145" t="n">
-        <v>5049200</v>
+        <v>2644700</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
-        <v>46239</v>
+        <v>46237</v>
       </c>
       <c r="B146" t="n">
-        <v>3.619999885559082</v>
+        <v>3.650000095367432</v>
       </c>
       <c r="C146" t="n">
-        <v>3.710000038146973</v>
+        <v>3.670000076293945</v>
       </c>
       <c r="D146" t="n">
-        <v>3.609999895095825</v>
+        <v>3.490000009536743</v>
       </c>
       <c r="E146" t="n">
-        <v>3.710000038146973</v>
+        <v>3.5</v>
       </c>
       <c r="F146" t="n">
-        <v>1946500</v>
+        <v>6262900</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
-        <v>46240</v>
+        <v>46238</v>
       </c>
       <c r="B147" t="n">
-        <v>3.569999933242798</v>
+        <v>3.680000066757202</v>
       </c>
       <c r="C147" t="n">
-        <v>3.619999885559082</v>
+        <v>3.779999971389771</v>
       </c>
       <c r="D147" t="n">
-        <v>3.519999980926514</v>
+        <v>3.589999914169312</v>
       </c>
       <c r="E147" t="n">
-        <v>3.569999933242798</v>
+        <v>3.660000085830688</v>
       </c>
       <c r="F147" t="n">
-        <v>2415500</v>
+        <v>5049200</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
-        <v>46241</v>
+        <v>46239</v>
       </c>
       <c r="B148" t="n">
-        <v>3.519999980926514</v>
+        <v>3.619999885559082</v>
       </c>
       <c r="C148" t="n">
-        <v>3.599999904632568</v>
+        <v>3.710000038146973</v>
       </c>
       <c r="D148" t="n">
-        <v>3.440000057220459</v>
+        <v>3.609999895095825</v>
       </c>
       <c r="E148" t="n">
-        <v>3.519999980926514</v>
+        <v>3.710000038146973</v>
       </c>
       <c r="F148" t="n">
-        <v>2618900</v>
+        <v>1946500</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
-        <v>46244</v>
+        <v>46240</v>
       </c>
       <c r="B149" t="n">
-        <v>3.410000085830688</v>
+        <v>3.569999933242798</v>
       </c>
       <c r="C149" t="n">
-        <v>3.5</v>
+        <v>3.619999885559082</v>
       </c>
       <c r="D149" t="n">
-        <v>3.390000104904175</v>
+        <v>3.519999980926514</v>
       </c>
       <c r="E149" t="n">
-        <v>3.450000047683716</v>
+        <v>3.569999933242798</v>
       </c>
       <c r="F149" t="n">
-        <v>2613600</v>
+        <v>2415500</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
-        <v>46245</v>
+        <v>46241</v>
       </c>
       <c r="B150" t="n">
-        <v>3.319999933242798</v>
+        <v>3.519999980926514</v>
       </c>
       <c r="C150" t="n">
+        <v>3.599999904632568</v>
+      </c>
+      <c r="D150" t="n">
         <v>3.440000057220459</v>
       </c>
-      <c r="D150" t="n">
-        <v>3.309999942779541</v>
-      </c>
       <c r="E150" t="n">
-        <v>3.369999885559082</v>
+        <v>3.519999980926514</v>
       </c>
       <c r="F150" t="n">
-        <v>5077500</v>
+        <v>2618900</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
-        <v>46246</v>
+        <v>46244</v>
       </c>
       <c r="B151" t="n">
-        <v>3.359999895095825</v>
+        <v>3.410000085830688</v>
       </c>
       <c r="C151" t="n">
-        <v>3.400000095367432</v>
+        <v>3.5</v>
       </c>
       <c r="D151" t="n">
-        <v>3.279999971389771</v>
+        <v>3.390000104904175</v>
       </c>
       <c r="E151" t="n">
-        <v>3.339999914169312</v>
+        <v>3.450000047683716</v>
       </c>
       <c r="F151" t="n">
-        <v>4336100</v>
+        <v>2613600</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
-        <v>46247</v>
+        <v>46245</v>
       </c>
       <c r="B152" t="n">
-        <v>3.450000047683716</v>
+        <v>3.319999933242798</v>
       </c>
       <c r="C152" t="n">
-        <v>3.470000028610229</v>
+        <v>3.440000057220459</v>
       </c>
       <c r="D152" t="n">
+        <v>3.309999942779541</v>
+      </c>
+      <c r="E152" t="n">
         <v>3.369999885559082</v>
       </c>
-      <c r="E152" t="n">
-        <v>3.390000104904175</v>
-      </c>
       <c r="F152" t="n">
-        <v>3777900</v>
+        <v>5077500</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B153" t="n">
+        <v>3.359999895095825</v>
+      </c>
+      <c r="C153" t="n">
+        <v>3.400000095367432</v>
+      </c>
+      <c r="D153" t="n">
+        <v>3.279999971389771</v>
+      </c>
+      <c r="E153" t="n">
+        <v>3.339999914169312</v>
+      </c>
+      <c r="F153" t="n">
+        <v>4336100</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="1" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B154" t="n">
+        <v>3.450000047683716</v>
+      </c>
+      <c r="C154" t="n">
+        <v>3.470000028610229</v>
+      </c>
+      <c r="D154" t="n">
+        <v>3.369999885559082</v>
+      </c>
+      <c r="E154" t="n">
+        <v>3.390000104904175</v>
+      </c>
+      <c r="F154" t="n">
+        <v>3777900</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="1" t="n">
         <v>46248</v>
       </c>
-      <c r="B153" t="n">
+      <c r="B155" t="n">
+        <v>3.160000085830688</v>
+      </c>
+      <c r="C155" t="n">
+        <v>3.420000076293945</v>
+      </c>
+      <c r="D155" t="n">
+        <v>3.089999914169312</v>
+      </c>
+      <c r="E155" t="n">
+        <v>3.410000085830688</v>
+      </c>
+      <c r="F155" t="n">
+        <v>12072100</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="1" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B156" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="C156" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="D156" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="E156" t="n">
         <v>3.16</v>
       </c>
-      <c r="C153" t="n">
-        <v>3.42</v>
-      </c>
-      <c r="D153" t="n">
-        <v>3.09</v>
-      </c>
-      <c r="E153" t="n">
-        <v>3.41</v>
-      </c>
-      <c r="F153" t="n">
-        <v>12069700</v>
+      <c r="F156" t="n">
+        <v>7840900</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-18 21:56 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -3309,242 +3309,242 @@
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="B145" t="n">
+        <v>3.650000095367432</v>
+      </c>
+      <c r="C145" t="n">
+        <v>3.670000076293945</v>
+      </c>
+      <c r="D145" t="n">
         <v>3.490000009536743</v>
       </c>
-      <c r="C145" t="n">
-        <v>3.539999961853027</v>
-      </c>
-      <c r="D145" t="n">
-        <v>3.380000114440918</v>
-      </c>
       <c r="E145" t="n">
-        <v>3.380000114440918</v>
+        <v>3.5</v>
       </c>
       <c r="F145" t="n">
-        <v>2644700</v>
+        <v>6262900</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B146" t="n">
-        <v>3.650000095367432</v>
+        <v>3.680000066757202</v>
       </c>
       <c r="C146" t="n">
-        <v>3.670000076293945</v>
+        <v>3.779999971389771</v>
       </c>
       <c r="D146" t="n">
-        <v>3.490000009536743</v>
+        <v>3.589999914169312</v>
       </c>
       <c r="E146" t="n">
-        <v>3.5</v>
+        <v>3.660000085830688</v>
       </c>
       <c r="F146" t="n">
-        <v>6262900</v>
+        <v>5049200</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="B147" t="n">
-        <v>3.680000066757202</v>
+        <v>3.619999885559082</v>
       </c>
       <c r="C147" t="n">
-        <v>3.779999971389771</v>
+        <v>3.710000038146973</v>
       </c>
       <c r="D147" t="n">
-        <v>3.589999914169312</v>
+        <v>3.609999895095825</v>
       </c>
       <c r="E147" t="n">
-        <v>3.660000085830688</v>
+        <v>3.710000038146973</v>
       </c>
       <c r="F147" t="n">
-        <v>5049200</v>
+        <v>1946500</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="B148" t="n">
+        <v>3.569999933242798</v>
+      </c>
+      <c r="C148" t="n">
         <v>3.619999885559082</v>
       </c>
-      <c r="C148" t="n">
-        <v>3.710000038146973</v>
-      </c>
       <c r="D148" t="n">
-        <v>3.609999895095825</v>
+        <v>3.519999980926514</v>
       </c>
       <c r="E148" t="n">
-        <v>3.710000038146973</v>
+        <v>3.569999933242798</v>
       </c>
       <c r="F148" t="n">
-        <v>1946500</v>
+        <v>2415500</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="B149" t="n">
-        <v>3.569999933242798</v>
+        <v>3.519999980926514</v>
       </c>
       <c r="C149" t="n">
-        <v>3.619999885559082</v>
+        <v>3.599999904632568</v>
       </c>
       <c r="D149" t="n">
+        <v>3.440000057220459</v>
+      </c>
+      <c r="E149" t="n">
         <v>3.519999980926514</v>
       </c>
-      <c r="E149" t="n">
-        <v>3.569999933242798</v>
-      </c>
       <c r="F149" t="n">
-        <v>2415500</v>
+        <v>2618900</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="B150" t="n">
-        <v>3.519999980926514</v>
+        <v>3.410000085830688</v>
       </c>
       <c r="C150" t="n">
-        <v>3.599999904632568</v>
+        <v>3.5</v>
       </c>
       <c r="D150" t="n">
-        <v>3.440000057220459</v>
+        <v>3.390000104904175</v>
       </c>
       <c r="E150" t="n">
-        <v>3.519999980926514</v>
+        <v>3.450000047683716</v>
       </c>
       <c r="F150" t="n">
-        <v>2618900</v>
+        <v>2613600</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="B151" t="n">
-        <v>3.410000085830688</v>
+        <v>3.319999933242798</v>
       </c>
       <c r="C151" t="n">
-        <v>3.5</v>
+        <v>3.440000057220459</v>
       </c>
       <c r="D151" t="n">
-        <v>3.390000104904175</v>
+        <v>3.309999942779541</v>
       </c>
       <c r="E151" t="n">
-        <v>3.450000047683716</v>
+        <v>3.369999885559082</v>
       </c>
       <c r="F151" t="n">
-        <v>2613600</v>
+        <v>5077500</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="B152" t="n">
-        <v>3.319999933242798</v>
+        <v>3.359999895095825</v>
       </c>
       <c r="C152" t="n">
-        <v>3.440000057220459</v>
+        <v>3.400000095367432</v>
       </c>
       <c r="D152" t="n">
-        <v>3.309999942779541</v>
+        <v>3.279999971389771</v>
       </c>
       <c r="E152" t="n">
-        <v>3.369999885559082</v>
+        <v>3.339999914169312</v>
       </c>
       <c r="F152" t="n">
-        <v>5077500</v>
+        <v>4336100</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="B153" t="n">
-        <v>3.359999895095825</v>
+        <v>3.450000047683716</v>
       </c>
       <c r="C153" t="n">
-        <v>3.400000095367432</v>
+        <v>3.470000028610229</v>
       </c>
       <c r="D153" t="n">
-        <v>3.279999971389771</v>
+        <v>3.369999885559082</v>
       </c>
       <c r="E153" t="n">
-        <v>3.339999914169312</v>
+        <v>3.390000104904175</v>
       </c>
       <c r="F153" t="n">
-        <v>4336100</v>
+        <v>3777900</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="B154" t="n">
-        <v>3.450000047683716</v>
+        <v>3.160000085830688</v>
       </c>
       <c r="C154" t="n">
-        <v>3.470000028610229</v>
+        <v>3.420000076293945</v>
       </c>
       <c r="D154" t="n">
-        <v>3.369999885559082</v>
+        <v>3.089999914169312</v>
       </c>
       <c r="E154" t="n">
-        <v>3.390000104904175</v>
+        <v>3.410000085830688</v>
       </c>
       <c r="F154" t="n">
-        <v>3777900</v>
+        <v>12072100</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="n">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="B155" t="n">
+        <v>3.130000114440918</v>
+      </c>
+      <c r="C155" t="n">
+        <v>3.210000038146973</v>
+      </c>
+      <c r="D155" t="n">
+        <v>3.049999952316284</v>
+      </c>
+      <c r="E155" t="n">
         <v>3.160000085830688</v>
       </c>
-      <c r="C155" t="n">
-        <v>3.420000076293945</v>
-      </c>
-      <c r="D155" t="n">
-        <v>3.089999914169312</v>
-      </c>
-      <c r="E155" t="n">
-        <v>3.410000085830688</v>
-      </c>
       <c r="F155" t="n">
-        <v>12072100</v>
+        <v>7840900</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="B156" t="n">
-        <v>3.13</v>
+        <v>3.14</v>
       </c>
       <c r="C156" t="n">
-        <v>3.21</v>
+        <v>3.19</v>
       </c>
       <c r="D156" t="n">
-        <v>3.05</v>
+        <v>3.1</v>
       </c>
       <c r="E156" t="n">
-        <v>3.16</v>
+        <v>3.12</v>
       </c>
       <c r="F156" t="n">
-        <v>7840900</v>
+        <v>2836700</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-19 21:59 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -3129,90 +3129,90 @@
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B136" t="n">
-        <v>3.160000085830688</v>
+        <v>3.140000104904175</v>
       </c>
       <c r="C136" t="n">
-        <v>3.200000047683716</v>
+        <v>3.170000076293945</v>
       </c>
       <c r="D136" t="n">
-        <v>3.079999923706055</v>
+        <v>3.089999914169312</v>
       </c>
       <c r="E136" t="n">
-        <v>3.079999923706055</v>
+        <v>3.130000114440918</v>
       </c>
       <c r="F136" t="n">
-        <v>2046300</v>
+        <v>2828500</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="B137" t="n">
-        <v>3.140000104904175</v>
+        <v>3.230000019073486</v>
       </c>
       <c r="C137" t="n">
-        <v>3.170000076293945</v>
+        <v>3.259999990463257</v>
       </c>
       <c r="D137" t="n">
-        <v>3.089999914169312</v>
+        <v>3.099999904632568</v>
       </c>
       <c r="E137" t="n">
         <v>3.130000114440918</v>
       </c>
       <c r="F137" t="n">
-        <v>2828500</v>
+        <v>3830200</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="B138" t="n">
-        <v>3.230000019073486</v>
+        <v>3.279999971389771</v>
       </c>
       <c r="C138" t="n">
-        <v>3.259999990463257</v>
+        <v>3.329999923706055</v>
       </c>
       <c r="D138" t="n">
-        <v>3.099999904632568</v>
+        <v>3.190000057220459</v>
       </c>
       <c r="E138" t="n">
-        <v>3.130000114440918</v>
+        <v>3.190000057220459</v>
       </c>
       <c r="F138" t="n">
-        <v>3830200</v>
+        <v>3736000</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="B139" t="n">
-        <v>3.279999971389771</v>
+        <v>3.259999990463257</v>
       </c>
       <c r="C139" t="n">
-        <v>3.329999923706055</v>
+        <v>3.269999980926514</v>
       </c>
       <c r="D139" t="n">
-        <v>3.190000057220459</v>
+        <v>3.210000038146973</v>
       </c>
       <c r="E139" t="n">
-        <v>3.190000057220459</v>
+        <v>3.259999990463257</v>
       </c>
       <c r="F139" t="n">
-        <v>3736000</v>
+        <v>1448700</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="B140" t="n">
-        <v>3.259999990463257</v>
+        <v>3.220000028610229</v>
       </c>
       <c r="C140" t="n">
         <v>3.269999980926514</v>
@@ -3221,330 +3221,330 @@
         <v>3.210000038146973</v>
       </c>
       <c r="E140" t="n">
-        <v>3.259999990463257</v>
+        <v>3.269999980926514</v>
       </c>
       <c r="F140" t="n">
-        <v>1448700</v>
+        <v>1750700</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B141" t="n">
-        <v>3.220000028610229</v>
+        <v>3.289999961853027</v>
       </c>
       <c r="C141" t="n">
+        <v>3.359999895095825</v>
+      </c>
+      <c r="D141" t="n">
         <v>3.269999980926514</v>
-      </c>
-      <c r="D141" t="n">
-        <v>3.210000038146973</v>
       </c>
       <c r="E141" t="n">
         <v>3.269999980926514</v>
       </c>
       <c r="F141" t="n">
-        <v>1750700</v>
+        <v>2817100</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B142" t="n">
-        <v>3.289999961853027</v>
+        <v>3.349999904632568</v>
       </c>
       <c r="C142" t="n">
-        <v>3.359999895095825</v>
+        <v>3.380000114440918</v>
       </c>
       <c r="D142" t="n">
-        <v>3.269999980926514</v>
+        <v>3.25</v>
       </c>
       <c r="E142" t="n">
-        <v>3.269999980926514</v>
+        <v>3.259999990463257</v>
       </c>
       <c r="F142" t="n">
-        <v>2817100</v>
+        <v>2720100</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B143" t="n">
-        <v>3.349999904632568</v>
+        <v>3.390000104904175</v>
       </c>
       <c r="C143" t="n">
-        <v>3.380000114440918</v>
+        <v>3.420000076293945</v>
       </c>
       <c r="D143" t="n">
-        <v>3.25</v>
+        <v>3.309999942779541</v>
       </c>
       <c r="E143" t="n">
-        <v>3.259999990463257</v>
+        <v>3.309999942779541</v>
       </c>
       <c r="F143" t="n">
-        <v>2720100</v>
+        <v>2171100</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
-        <v>46233</v>
+        <v>46237</v>
       </c>
       <c r="B144" t="n">
-        <v>3.390000104904175</v>
+        <v>3.650000095367432</v>
       </c>
       <c r="C144" t="n">
-        <v>3.420000076293945</v>
+        <v>3.670000076293945</v>
       </c>
       <c r="D144" t="n">
-        <v>3.309999942779541</v>
+        <v>3.490000009536743</v>
       </c>
       <c r="E144" t="n">
-        <v>3.309999942779541</v>
+        <v>3.5</v>
       </c>
       <c r="F144" t="n">
-        <v>2171100</v>
+        <v>6262900</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B145" t="n">
-        <v>3.650000095367432</v>
+        <v>3.680000066757202</v>
       </c>
       <c r="C145" t="n">
-        <v>3.670000076293945</v>
+        <v>3.779999971389771</v>
       </c>
       <c r="D145" t="n">
-        <v>3.490000009536743</v>
+        <v>3.589999914169312</v>
       </c>
       <c r="E145" t="n">
-        <v>3.5</v>
+        <v>3.660000085830688</v>
       </c>
       <c r="F145" t="n">
-        <v>6262900</v>
+        <v>5049200</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="B146" t="n">
-        <v>3.680000066757202</v>
+        <v>3.619999885559082</v>
       </c>
       <c r="C146" t="n">
-        <v>3.779999971389771</v>
+        <v>3.710000038146973</v>
       </c>
       <c r="D146" t="n">
-        <v>3.589999914169312</v>
+        <v>3.609999895095825</v>
       </c>
       <c r="E146" t="n">
-        <v>3.660000085830688</v>
+        <v>3.710000038146973</v>
       </c>
       <c r="F146" t="n">
-        <v>5049200</v>
+        <v>1946500</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="B147" t="n">
+        <v>3.569999933242798</v>
+      </c>
+      <c r="C147" t="n">
         <v>3.619999885559082</v>
       </c>
-      <c r="C147" t="n">
-        <v>3.710000038146973</v>
-      </c>
       <c r="D147" t="n">
-        <v>3.609999895095825</v>
+        <v>3.519999980926514</v>
       </c>
       <c r="E147" t="n">
-        <v>3.710000038146973</v>
+        <v>3.569999933242798</v>
       </c>
       <c r="F147" t="n">
-        <v>1946500</v>
+        <v>2415500</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="B148" t="n">
-        <v>3.569999933242798</v>
+        <v>3.519999980926514</v>
       </c>
       <c r="C148" t="n">
-        <v>3.619999885559082</v>
+        <v>3.599999904632568</v>
       </c>
       <c r="D148" t="n">
+        <v>3.440000057220459</v>
+      </c>
+      <c r="E148" t="n">
         <v>3.519999980926514</v>
       </c>
-      <c r="E148" t="n">
-        <v>3.569999933242798</v>
-      </c>
       <c r="F148" t="n">
-        <v>2415500</v>
+        <v>2618900</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="B149" t="n">
-        <v>3.519999980926514</v>
+        <v>3.410000085830688</v>
       </c>
       <c r="C149" t="n">
-        <v>3.599999904632568</v>
+        <v>3.5</v>
       </c>
       <c r="D149" t="n">
-        <v>3.440000057220459</v>
+        <v>3.390000104904175</v>
       </c>
       <c r="E149" t="n">
-        <v>3.519999980926514</v>
+        <v>3.450000047683716</v>
       </c>
       <c r="F149" t="n">
-        <v>2618900</v>
+        <v>2613600</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="B150" t="n">
-        <v>3.410000085830688</v>
+        <v>3.319999933242798</v>
       </c>
       <c r="C150" t="n">
-        <v>3.5</v>
+        <v>3.440000057220459</v>
       </c>
       <c r="D150" t="n">
-        <v>3.390000104904175</v>
+        <v>3.309999942779541</v>
       </c>
       <c r="E150" t="n">
-        <v>3.450000047683716</v>
+        <v>3.369999885559082</v>
       </c>
       <c r="F150" t="n">
-        <v>2613600</v>
+        <v>5077500</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="B151" t="n">
-        <v>3.319999933242798</v>
+        <v>3.359999895095825</v>
       </c>
       <c r="C151" t="n">
-        <v>3.440000057220459</v>
+        <v>3.400000095367432</v>
       </c>
       <c r="D151" t="n">
-        <v>3.309999942779541</v>
+        <v>3.279999971389771</v>
       </c>
       <c r="E151" t="n">
-        <v>3.369999885559082</v>
+        <v>3.339999914169312</v>
       </c>
       <c r="F151" t="n">
-        <v>5077500</v>
+        <v>4336100</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="B152" t="n">
-        <v>3.359999895095825</v>
+        <v>3.450000047683716</v>
       </c>
       <c r="C152" t="n">
-        <v>3.400000095367432</v>
+        <v>3.470000028610229</v>
       </c>
       <c r="D152" t="n">
-        <v>3.279999971389771</v>
+        <v>3.369999885559082</v>
       </c>
       <c r="E152" t="n">
-        <v>3.339999914169312</v>
+        <v>3.390000104904175</v>
       </c>
       <c r="F152" t="n">
-        <v>4336100</v>
+        <v>3777900</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="B153" t="n">
-        <v>3.450000047683716</v>
+        <v>3.160000085830688</v>
       </c>
       <c r="C153" t="n">
-        <v>3.470000028610229</v>
+        <v>3.420000076293945</v>
       </c>
       <c r="D153" t="n">
-        <v>3.369999885559082</v>
+        <v>3.089999914169312</v>
       </c>
       <c r="E153" t="n">
-        <v>3.390000104904175</v>
+        <v>3.410000085830688</v>
       </c>
       <c r="F153" t="n">
-        <v>3777900</v>
+        <v>12072100</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="n">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="B154" t="n">
+        <v>3.130000114440918</v>
+      </c>
+      <c r="C154" t="n">
+        <v>3.210000038146973</v>
+      </c>
+      <c r="D154" t="n">
+        <v>3.049999952316284</v>
+      </c>
+      <c r="E154" t="n">
         <v>3.160000085830688</v>
       </c>
-      <c r="C154" t="n">
-        <v>3.420000076293945</v>
-      </c>
-      <c r="D154" t="n">
-        <v>3.089999914169312</v>
-      </c>
-      <c r="E154" t="n">
-        <v>3.410000085830688</v>
-      </c>
       <c r="F154" t="n">
-        <v>12072100</v>
+        <v>7840900</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="B155" t="n">
-        <v>3.130000114440918</v>
+        <v>3.140000104904175</v>
       </c>
       <c r="C155" t="n">
-        <v>3.210000038146973</v>
+        <v>3.190000057220459</v>
       </c>
       <c r="D155" t="n">
-        <v>3.049999952316284</v>
+        <v>3.099999904632568</v>
       </c>
       <c r="E155" t="n">
-        <v>3.160000085830688</v>
+        <v>3.119999885559082</v>
       </c>
       <c r="F155" t="n">
-        <v>7840900</v>
+        <v>2836700</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="B156" t="n">
-        <v>3.14</v>
+        <v>3.25</v>
       </c>
       <c r="C156" t="n">
-        <v>3.19</v>
+        <v>3.28</v>
       </c>
       <c r="D156" t="n">
-        <v>3.1</v>
+        <v>3.15</v>
       </c>
       <c r="E156" t="n">
-        <v>3.12</v>
+        <v>3.17</v>
       </c>
       <c r="F156" t="n">
-        <v>2836700</v>
+        <v>3313800</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-20 22:01 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F156"/>
+  <dimension ref="A1:F158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3129,90 +3129,90 @@
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
-        <v>46224</v>
+        <v>46223</v>
       </c>
       <c r="B136" t="n">
-        <v>3.140000104904175</v>
+        <v>3.160000085830688</v>
       </c>
       <c r="C136" t="n">
-        <v>3.170000076293945</v>
+        <v>3.200000047683716</v>
       </c>
       <c r="D136" t="n">
-        <v>3.089999914169312</v>
+        <v>3.079999923706055</v>
       </c>
       <c r="E136" t="n">
-        <v>3.130000114440918</v>
+        <v>3.079999923706055</v>
       </c>
       <c r="F136" t="n">
-        <v>2828500</v>
+        <v>2046300</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
-        <v>46225</v>
+        <v>46224</v>
       </c>
       <c r="B137" t="n">
-        <v>3.230000019073486</v>
+        <v>3.140000104904175</v>
       </c>
       <c r="C137" t="n">
-        <v>3.259999990463257</v>
+        <v>3.170000076293945</v>
       </c>
       <c r="D137" t="n">
-        <v>3.099999904632568</v>
+        <v>3.089999914169312</v>
       </c>
       <c r="E137" t="n">
         <v>3.130000114440918</v>
       </c>
       <c r="F137" t="n">
-        <v>3830200</v>
+        <v>2828500</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
-        <v>46226</v>
+        <v>46225</v>
       </c>
       <c r="B138" t="n">
-        <v>3.279999971389771</v>
+        <v>3.230000019073486</v>
       </c>
       <c r="C138" t="n">
-        <v>3.329999923706055</v>
+        <v>3.259999990463257</v>
       </c>
       <c r="D138" t="n">
-        <v>3.190000057220459</v>
+        <v>3.099999904632568</v>
       </c>
       <c r="E138" t="n">
-        <v>3.190000057220459</v>
+        <v>3.130000114440918</v>
       </c>
       <c r="F138" t="n">
-        <v>3736000</v>
+        <v>3830200</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
-        <v>46227</v>
+        <v>46226</v>
       </c>
       <c r="B139" t="n">
-        <v>3.259999990463257</v>
+        <v>3.279999971389771</v>
       </c>
       <c r="C139" t="n">
-        <v>3.269999980926514</v>
+        <v>3.329999923706055</v>
       </c>
       <c r="D139" t="n">
-        <v>3.210000038146973</v>
+        <v>3.190000057220459</v>
       </c>
       <c r="E139" t="n">
-        <v>3.259999990463257</v>
+        <v>3.190000057220459</v>
       </c>
       <c r="F139" t="n">
-        <v>1448700</v>
+        <v>3736000</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
-        <v>46230</v>
+        <v>46227</v>
       </c>
       <c r="B140" t="n">
-        <v>3.220000028610229</v>
+        <v>3.259999990463257</v>
       </c>
       <c r="C140" t="n">
         <v>3.269999980926514</v>
@@ -3221,330 +3221,370 @@
         <v>3.210000038146973</v>
       </c>
       <c r="E140" t="n">
-        <v>3.269999980926514</v>
+        <v>3.259999990463257</v>
       </c>
       <c r="F140" t="n">
-        <v>1750700</v>
+        <v>1448700</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
-        <v>46231</v>
+        <v>46230</v>
       </c>
       <c r="B141" t="n">
-        <v>3.289999961853027</v>
+        <v>3.220000028610229</v>
       </c>
       <c r="C141" t="n">
-        <v>3.359999895095825</v>
+        <v>3.269999980926514</v>
       </c>
       <c r="D141" t="n">
-        <v>3.269999980926514</v>
+        <v>3.210000038146973</v>
       </c>
       <c r="E141" t="n">
         <v>3.269999980926514</v>
       </c>
       <c r="F141" t="n">
-        <v>2817100</v>
+        <v>1750700</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
-        <v>46232</v>
+        <v>46231</v>
       </c>
       <c r="B142" t="n">
-        <v>3.349999904632568</v>
+        <v>3.289999961853027</v>
       </c>
       <c r="C142" t="n">
-        <v>3.380000114440918</v>
+        <v>3.359999895095825</v>
       </c>
       <c r="D142" t="n">
-        <v>3.25</v>
+        <v>3.269999980926514</v>
       </c>
       <c r="E142" t="n">
-        <v>3.259999990463257</v>
+        <v>3.269999980926514</v>
       </c>
       <c r="F142" t="n">
-        <v>2720100</v>
+        <v>2817100</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
-        <v>46233</v>
+        <v>46232</v>
       </c>
       <c r="B143" t="n">
-        <v>3.390000104904175</v>
+        <v>3.349999904632568</v>
       </c>
       <c r="C143" t="n">
-        <v>3.420000076293945</v>
+        <v>3.380000114440918</v>
       </c>
       <c r="D143" t="n">
-        <v>3.309999942779541</v>
+        <v>3.25</v>
       </c>
       <c r="E143" t="n">
-        <v>3.309999942779541</v>
+        <v>3.259999990463257</v>
       </c>
       <c r="F143" t="n">
-        <v>2171100</v>
+        <v>2720100</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
-        <v>46237</v>
+        <v>46233</v>
       </c>
       <c r="B144" t="n">
-        <v>3.650000095367432</v>
+        <v>3.390000104904175</v>
       </c>
       <c r="C144" t="n">
-        <v>3.670000076293945</v>
+        <v>3.420000076293945</v>
       </c>
       <c r="D144" t="n">
-        <v>3.490000009536743</v>
+        <v>3.309999942779541</v>
       </c>
       <c r="E144" t="n">
-        <v>3.5</v>
+        <v>3.309999942779541</v>
       </c>
       <c r="F144" t="n">
-        <v>6262900</v>
+        <v>2171100</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
-        <v>46238</v>
+        <v>46237</v>
       </c>
       <c r="B145" t="n">
-        <v>3.680000066757202</v>
+        <v>3.650000095367432</v>
       </c>
       <c r="C145" t="n">
-        <v>3.779999971389771</v>
+        <v>3.670000076293945</v>
       </c>
       <c r="D145" t="n">
-        <v>3.589999914169312</v>
+        <v>3.490000009536743</v>
       </c>
       <c r="E145" t="n">
-        <v>3.660000085830688</v>
+        <v>3.5</v>
       </c>
       <c r="F145" t="n">
-        <v>5049200</v>
+        <v>6262900</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
-        <v>46239</v>
+        <v>46238</v>
       </c>
       <c r="B146" t="n">
-        <v>3.619999885559082</v>
+        <v>3.680000066757202</v>
       </c>
       <c r="C146" t="n">
-        <v>3.710000038146973</v>
+        <v>3.779999971389771</v>
       </c>
       <c r="D146" t="n">
-        <v>3.609999895095825</v>
+        <v>3.589999914169312</v>
       </c>
       <c r="E146" t="n">
-        <v>3.710000038146973</v>
+        <v>3.660000085830688</v>
       </c>
       <c r="F146" t="n">
-        <v>1946500</v>
+        <v>5049200</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
-        <v>46240</v>
+        <v>46239</v>
       </c>
       <c r="B147" t="n">
-        <v>3.569999933242798</v>
+        <v>3.619999885559082</v>
       </c>
       <c r="C147" t="n">
-        <v>3.619999885559082</v>
+        <v>3.710000038146973</v>
       </c>
       <c r="D147" t="n">
-        <v>3.519999980926514</v>
+        <v>3.609999895095825</v>
       </c>
       <c r="E147" t="n">
-        <v>3.569999933242798</v>
+        <v>3.710000038146973</v>
       </c>
       <c r="F147" t="n">
-        <v>2415500</v>
+        <v>1946500</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
-        <v>46241</v>
+        <v>46240</v>
       </c>
       <c r="B148" t="n">
+        <v>3.569999933242798</v>
+      </c>
+      <c r="C148" t="n">
+        <v>3.619999885559082</v>
+      </c>
+      <c r="D148" t="n">
         <v>3.519999980926514</v>
       </c>
-      <c r="C148" t="n">
-        <v>3.599999904632568</v>
-      </c>
-      <c r="D148" t="n">
-        <v>3.440000057220459</v>
-      </c>
       <c r="E148" t="n">
-        <v>3.519999980926514</v>
+        <v>3.569999933242798</v>
       </c>
       <c r="F148" t="n">
-        <v>2618900</v>
+        <v>2415500</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
-        <v>46244</v>
+        <v>46241</v>
       </c>
       <c r="B149" t="n">
-        <v>3.410000085830688</v>
+        <v>3.519999980926514</v>
       </c>
       <c r="C149" t="n">
-        <v>3.5</v>
+        <v>3.599999904632568</v>
       </c>
       <c r="D149" t="n">
-        <v>3.390000104904175</v>
+        <v>3.440000057220459</v>
       </c>
       <c r="E149" t="n">
-        <v>3.450000047683716</v>
+        <v>3.519999980926514</v>
       </c>
       <c r="F149" t="n">
-        <v>2613600</v>
+        <v>2618900</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
-        <v>46245</v>
+        <v>46244</v>
       </c>
       <c r="B150" t="n">
-        <v>3.319999933242798</v>
+        <v>3.410000085830688</v>
       </c>
       <c r="C150" t="n">
-        <v>3.440000057220459</v>
+        <v>3.5</v>
       </c>
       <c r="D150" t="n">
-        <v>3.309999942779541</v>
+        <v>3.390000104904175</v>
       </c>
       <c r="E150" t="n">
-        <v>3.369999885559082</v>
+        <v>3.450000047683716</v>
       </c>
       <c r="F150" t="n">
-        <v>5077500</v>
+        <v>2613600</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
-        <v>46246</v>
+        <v>46245</v>
       </c>
       <c r="B151" t="n">
-        <v>3.359999895095825</v>
+        <v>3.319999933242798</v>
       </c>
       <c r="C151" t="n">
-        <v>3.400000095367432</v>
+        <v>3.440000057220459</v>
       </c>
       <c r="D151" t="n">
-        <v>3.279999971389771</v>
+        <v>3.309999942779541</v>
       </c>
       <c r="E151" t="n">
-        <v>3.339999914169312</v>
+        <v>3.369999885559082</v>
       </c>
       <c r="F151" t="n">
-        <v>4336100</v>
+        <v>5077500</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
-        <v>46247</v>
+        <v>46246</v>
       </c>
       <c r="B152" t="n">
-        <v>3.450000047683716</v>
+        <v>3.359999895095825</v>
       </c>
       <c r="C152" t="n">
-        <v>3.470000028610229</v>
+        <v>3.400000095367432</v>
       </c>
       <c r="D152" t="n">
-        <v>3.369999885559082</v>
+        <v>3.279999971389771</v>
       </c>
       <c r="E152" t="n">
-        <v>3.390000104904175</v>
+        <v>3.339999914169312</v>
       </c>
       <c r="F152" t="n">
-        <v>3777900</v>
+        <v>4336100</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="B153" t="n">
-        <v>3.160000085830688</v>
+        <v>3.450000047683716</v>
       </c>
       <c r="C153" t="n">
-        <v>3.420000076293945</v>
+        <v>3.470000028610229</v>
       </c>
       <c r="D153" t="n">
-        <v>3.089999914169312</v>
+        <v>3.369999885559082</v>
       </c>
       <c r="E153" t="n">
-        <v>3.410000085830688</v>
+        <v>3.390000104904175</v>
       </c>
       <c r="F153" t="n">
-        <v>12072100</v>
+        <v>3777900</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="n">
-        <v>46251</v>
+        <v>46248</v>
       </c>
       <c r="B154" t="n">
-        <v>3.130000114440918</v>
+        <v>3.160000085830688</v>
       </c>
       <c r="C154" t="n">
-        <v>3.210000038146973</v>
+        <v>3.420000076293945</v>
       </c>
       <c r="D154" t="n">
-        <v>3.049999952316284</v>
+        <v>3.089999914169312</v>
       </c>
       <c r="E154" t="n">
-        <v>3.160000085830688</v>
+        <v>3.410000085830688</v>
       </c>
       <c r="F154" t="n">
-        <v>7840900</v>
+        <v>12072100</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="n">
-        <v>46252</v>
+        <v>46251</v>
       </c>
       <c r="B155" t="n">
-        <v>3.140000104904175</v>
+        <v>3.130000114440918</v>
       </c>
       <c r="C155" t="n">
-        <v>3.190000057220459</v>
+        <v>3.210000038146973</v>
       </c>
       <c r="D155" t="n">
-        <v>3.099999904632568</v>
+        <v>3.049999952316284</v>
       </c>
       <c r="E155" t="n">
-        <v>3.119999885559082</v>
+        <v>3.160000085830688</v>
       </c>
       <c r="F155" t="n">
-        <v>2836700</v>
+        <v>7840900</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B156" t="n">
+        <v>3.140000104904175</v>
+      </c>
+      <c r="C156" t="n">
+        <v>3.190000057220459</v>
+      </c>
+      <c r="D156" t="n">
+        <v>3.099999904632568</v>
+      </c>
+      <c r="E156" t="n">
+        <v>3.119999885559082</v>
+      </c>
+      <c r="F156" t="n">
+        <v>2836700</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="1" t="n">
         <v>46253</v>
       </c>
-      <c r="B156" t="n">
+      <c r="B157" t="n">
         <v>3.25</v>
       </c>
-      <c r="C156" t="n">
-        <v>3.28</v>
-      </c>
-      <c r="D156" t="n">
-        <v>3.15</v>
-      </c>
-      <c r="E156" t="n">
-        <v>3.17</v>
-      </c>
-      <c r="F156" t="n">
+      <c r="C157" t="n">
+        <v>3.279999971389771</v>
+      </c>
+      <c r="D157" t="n">
+        <v>3.150000095367432</v>
+      </c>
+      <c r="E157" t="n">
+        <v>3.170000076293945</v>
+      </c>
+      <c r="F157" t="n">
         <v>3313800</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="1" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B158" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="C158" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="D158" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="E158" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F158" t="n">
+        <v>5941100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-21 21:57 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F158"/>
+  <dimension ref="A1:F160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3309,282 +3309,322 @@
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
-        <v>46237</v>
+        <v>46234</v>
       </c>
       <c r="B145" t="n">
-        <v>3.650000095367432</v>
+        <v>3.490000009536743</v>
       </c>
       <c r="C145" t="n">
-        <v>3.670000076293945</v>
+        <v>3.539999961853027</v>
       </c>
       <c r="D145" t="n">
-        <v>3.490000009536743</v>
+        <v>3.380000114440918</v>
       </c>
       <c r="E145" t="n">
-        <v>3.5</v>
+        <v>3.380000114440918</v>
       </c>
       <c r="F145" t="n">
-        <v>6262900</v>
+        <v>2644700</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
-        <v>46238</v>
+        <v>46237</v>
       </c>
       <c r="B146" t="n">
-        <v>3.680000066757202</v>
+        <v>3.650000095367432</v>
       </c>
       <c r="C146" t="n">
-        <v>3.779999971389771</v>
+        <v>3.670000076293945</v>
       </c>
       <c r="D146" t="n">
-        <v>3.589999914169312</v>
+        <v>3.490000009536743</v>
       </c>
       <c r="E146" t="n">
-        <v>3.660000085830688</v>
+        <v>3.5</v>
       </c>
       <c r="F146" t="n">
-        <v>5049200</v>
+        <v>6262900</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
-        <v>46239</v>
+        <v>46238</v>
       </c>
       <c r="B147" t="n">
-        <v>3.619999885559082</v>
+        <v>3.680000066757202</v>
       </c>
       <c r="C147" t="n">
-        <v>3.710000038146973</v>
+        <v>3.779999971389771</v>
       </c>
       <c r="D147" t="n">
-        <v>3.609999895095825</v>
+        <v>3.589999914169312</v>
       </c>
       <c r="E147" t="n">
-        <v>3.710000038146973</v>
+        <v>3.660000085830688</v>
       </c>
       <c r="F147" t="n">
-        <v>1946500</v>
+        <v>5049200</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
-        <v>46240</v>
+        <v>46239</v>
       </c>
       <c r="B148" t="n">
-        <v>3.569999933242798</v>
+        <v>3.619999885559082</v>
       </c>
       <c r="C148" t="n">
-        <v>3.619999885559082</v>
+        <v>3.710000038146973</v>
       </c>
       <c r="D148" t="n">
-        <v>3.519999980926514</v>
+        <v>3.609999895095825</v>
       </c>
       <c r="E148" t="n">
-        <v>3.569999933242798</v>
+        <v>3.710000038146973</v>
       </c>
       <c r="F148" t="n">
-        <v>2415500</v>
+        <v>1946500</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
-        <v>46241</v>
+        <v>46240</v>
       </c>
       <c r="B149" t="n">
+        <v>3.569999933242798</v>
+      </c>
+      <c r="C149" t="n">
+        <v>3.619999885559082</v>
+      </c>
+      <c r="D149" t="n">
         <v>3.519999980926514</v>
       </c>
-      <c r="C149" t="n">
-        <v>3.599999904632568</v>
-      </c>
-      <c r="D149" t="n">
-        <v>3.440000057220459</v>
-      </c>
       <c r="E149" t="n">
-        <v>3.519999980926514</v>
+        <v>3.569999933242798</v>
       </c>
       <c r="F149" t="n">
-        <v>2618900</v>
+        <v>2415500</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
-        <v>46244</v>
+        <v>46241</v>
       </c>
       <c r="B150" t="n">
-        <v>3.410000085830688</v>
+        <v>3.519999980926514</v>
       </c>
       <c r="C150" t="n">
-        <v>3.5</v>
+        <v>3.599999904632568</v>
       </c>
       <c r="D150" t="n">
-        <v>3.390000104904175</v>
+        <v>3.440000057220459</v>
       </c>
       <c r="E150" t="n">
-        <v>3.450000047683716</v>
+        <v>3.519999980926514</v>
       </c>
       <c r="F150" t="n">
-        <v>2613600</v>
+        <v>2618900</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
-        <v>46245</v>
+        <v>46244</v>
       </c>
       <c r="B151" t="n">
-        <v>3.319999933242798</v>
+        <v>3.410000085830688</v>
       </c>
       <c r="C151" t="n">
-        <v>3.440000057220459</v>
+        <v>3.5</v>
       </c>
       <c r="D151" t="n">
-        <v>3.309999942779541</v>
+        <v>3.390000104904175</v>
       </c>
       <c r="E151" t="n">
-        <v>3.369999885559082</v>
+        <v>3.450000047683716</v>
       </c>
       <c r="F151" t="n">
-        <v>5077500</v>
+        <v>2613600</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
-        <v>46246</v>
+        <v>46245</v>
       </c>
       <c r="B152" t="n">
-        <v>3.359999895095825</v>
+        <v>3.319999933242798</v>
       </c>
       <c r="C152" t="n">
-        <v>3.400000095367432</v>
+        <v>3.440000057220459</v>
       </c>
       <c r="D152" t="n">
-        <v>3.279999971389771</v>
+        <v>3.309999942779541</v>
       </c>
       <c r="E152" t="n">
-        <v>3.339999914169312</v>
+        <v>3.369999885559082</v>
       </c>
       <c r="F152" t="n">
-        <v>4336100</v>
+        <v>5077500</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
-        <v>46247</v>
+        <v>46246</v>
       </c>
       <c r="B153" t="n">
-        <v>3.450000047683716</v>
+        <v>3.359999895095825</v>
       </c>
       <c r="C153" t="n">
-        <v>3.470000028610229</v>
+        <v>3.400000095367432</v>
       </c>
       <c r="D153" t="n">
-        <v>3.369999885559082</v>
+        <v>3.279999971389771</v>
       </c>
       <c r="E153" t="n">
-        <v>3.390000104904175</v>
+        <v>3.339999914169312</v>
       </c>
       <c r="F153" t="n">
-        <v>3777900</v>
+        <v>4336100</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="B154" t="n">
-        <v>3.160000085830688</v>
+        <v>3.450000047683716</v>
       </c>
       <c r="C154" t="n">
-        <v>3.420000076293945</v>
+        <v>3.470000028610229</v>
       </c>
       <c r="D154" t="n">
-        <v>3.089999914169312</v>
+        <v>3.369999885559082</v>
       </c>
       <c r="E154" t="n">
-        <v>3.410000085830688</v>
+        <v>3.390000104904175</v>
       </c>
       <c r="F154" t="n">
-        <v>12072100</v>
+        <v>3777900</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="n">
-        <v>46251</v>
+        <v>46248</v>
       </c>
       <c r="B155" t="n">
-        <v>3.130000114440918</v>
+        <v>3.160000085830688</v>
       </c>
       <c r="C155" t="n">
-        <v>3.210000038146973</v>
+        <v>3.420000076293945</v>
       </c>
       <c r="D155" t="n">
-        <v>3.049999952316284</v>
+        <v>3.089999914169312</v>
       </c>
       <c r="E155" t="n">
-        <v>3.160000085830688</v>
+        <v>3.410000085830688</v>
       </c>
       <c r="F155" t="n">
-        <v>7840900</v>
+        <v>12072100</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
-        <v>46252</v>
+        <v>46251</v>
       </c>
       <c r="B156" t="n">
-        <v>3.140000104904175</v>
+        <v>3.130000114440918</v>
       </c>
       <c r="C156" t="n">
-        <v>3.190000057220459</v>
+        <v>3.210000038146973</v>
       </c>
       <c r="D156" t="n">
-        <v>3.099999904632568</v>
+        <v>3.049999952316284</v>
       </c>
       <c r="E156" t="n">
-        <v>3.119999885559082</v>
+        <v>3.160000085830688</v>
       </c>
       <c r="F156" t="n">
-        <v>2836700</v>
+        <v>7840900</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="n">
-        <v>46253</v>
+        <v>46252</v>
       </c>
       <c r="B157" t="n">
-        <v>3.25</v>
+        <v>3.140000104904175</v>
       </c>
       <c r="C157" t="n">
-        <v>3.279999971389771</v>
+        <v>3.190000057220459</v>
       </c>
       <c r="D157" t="n">
-        <v>3.150000095367432</v>
+        <v>3.099999904632568</v>
       </c>
       <c r="E157" t="n">
-        <v>3.170000076293945</v>
+        <v>3.119999885559082</v>
       </c>
       <c r="F157" t="n">
-        <v>3313800</v>
+        <v>2836700</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B158" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="C158" t="n">
+        <v>3.279999971389771</v>
+      </c>
+      <c r="D158" t="n">
+        <v>3.150000095367432</v>
+      </c>
+      <c r="E158" t="n">
+        <v>3.170000076293945</v>
+      </c>
+      <c r="F158" t="n">
+        <v>3313800</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="1" t="n">
         <v>46254</v>
       </c>
-      <c r="B158" t="n">
-        <v>3.19</v>
-      </c>
-      <c r="C158" t="n">
-        <v>3.27</v>
-      </c>
-      <c r="D158" t="n">
-        <v>3.07</v>
-      </c>
-      <c r="E158" t="n">
+      <c r="B159" t="n">
+        <v>3.190000057220459</v>
+      </c>
+      <c r="C159" t="n">
+        <v>3.269999980926514</v>
+      </c>
+      <c r="D159" t="n">
+        <v>3.069999933242798</v>
+      </c>
+      <c r="E159" t="n">
         <v>3.25</v>
       </c>
-      <c r="F158" t="n">
+      <c r="F159" t="n">
         <v>5941100</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="1" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B160" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="C160" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="D160" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="E160" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="F160" t="n">
+        <v>9016400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-24 22:02 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F160"/>
+  <dimension ref="A1:F161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3612,19 +3612,39 @@
         <v>46255</v>
       </c>
       <c r="B160" t="n">
-        <v>3.22</v>
+        <v>3.220000028610229</v>
       </c>
       <c r="C160" t="n">
-        <v>3.29</v>
+        <v>3.289999961853027</v>
       </c>
       <c r="D160" t="n">
-        <v>3.17</v>
+        <v>3.170000076293945</v>
       </c>
       <c r="E160" t="n">
-        <v>3.18</v>
+        <v>3.180000066757202</v>
       </c>
       <c r="F160" t="n">
         <v>9016400</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="1" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B161" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="C161" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="D161" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="E161" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F161" t="n">
+        <v>2932200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-25 22:01 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F161"/>
+  <dimension ref="A1:F162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3632,19 +3632,39 @@
         <v>46258</v>
       </c>
       <c r="B161" t="n">
-        <v>3.23</v>
+        <v>3.230000019073486</v>
       </c>
       <c r="C161" t="n">
-        <v>3.28</v>
+        <v>3.279999971389771</v>
       </c>
       <c r="D161" t="n">
-        <v>3.16</v>
+        <v>3.160000085830688</v>
       </c>
       <c r="E161" t="n">
-        <v>3.2</v>
+        <v>3.200000047683716</v>
       </c>
       <c r="F161" t="n">
         <v>2932200</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B162" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="C162" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="D162" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E162" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F162" t="n">
+        <v>4436900</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-27 00:39 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F162"/>
+  <dimension ref="A1:F163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3652,19 +3652,39 @@
         <v>46259</v>
       </c>
       <c r="B162" t="n">
-        <v>3.33</v>
+        <v>3.329999923706055</v>
       </c>
       <c r="C162" t="n">
-        <v>3.37</v>
+        <v>3.369999885559082</v>
       </c>
       <c r="D162" t="n">
-        <v>3.2</v>
+        <v>3.200000047683716</v>
       </c>
       <c r="E162" t="n">
-        <v>3.2</v>
+        <v>3.200000047683716</v>
       </c>
       <c r="F162" t="n">
         <v>4436900</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="1" t="n">
+        <v>46260</v>
+      </c>
+      <c r="B163" t="n">
+        <v>3.279999971389771</v>
+      </c>
+      <c r="C163" t="n">
+        <v>3.380000114440918</v>
+      </c>
+      <c r="D163" t="n">
+        <v>3.240000009536743</v>
+      </c>
+      <c r="E163" t="n">
+        <v>3.349999904632568</v>
+      </c>
+      <c r="F163" t="n">
+        <v>1940200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-28 05:41 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F163"/>
+  <dimension ref="A1:F164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3684,7 +3684,27 @@
         <v>3.349999904632568</v>
       </c>
       <c r="F163" t="n">
-        <v>1940200</v>
+        <v>1973900</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="1" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B164" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="C164" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="D164" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E164" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F164" t="n">
+        <v>2085400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-28 18:49 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F164"/>
+  <dimension ref="A1:F165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3692,19 +3692,39 @@
         <v>46261</v>
       </c>
       <c r="B164" t="n">
-        <v>3.3</v>
+        <v>3.299999952316284</v>
       </c>
       <c r="C164" t="n">
-        <v>3.34</v>
+        <v>3.339999914169312</v>
       </c>
       <c r="D164" t="n">
-        <v>3.24</v>
+        <v>3.240000009536743</v>
       </c>
       <c r="E164" t="n">
-        <v>3.27</v>
+        <v>3.269999980926514</v>
       </c>
       <c r="F164" t="n">
         <v>2085400</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="1" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B165" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="C165" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="D165" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="E165" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="F165" t="n">
+        <v>1732200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-28 21:37 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -3712,10 +3712,10 @@
         <v>46262</v>
       </c>
       <c r="B165" t="n">
-        <v>3.31</v>
+        <v>3.35</v>
       </c>
       <c r="C165" t="n">
-        <v>3.34</v>
+        <v>3.35</v>
       </c>
       <c r="D165" t="n">
         <v>3.27</v>
@@ -3724,7 +3724,7 @@
         <v>3.29</v>
       </c>
       <c r="F165" t="n">
-        <v>1732200</v>
+        <v>2352400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-08-29 03:25 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -3711,18 +3711,10 @@
       <c r="A165" s="1" t="n">
         <v>46262</v>
       </c>
-      <c r="B165" t="n">
-        <v>3.35</v>
-      </c>
-      <c r="C165" t="n">
-        <v>3.35</v>
-      </c>
-      <c r="D165" t="n">
-        <v>3.27</v>
-      </c>
-      <c r="E165" t="n">
-        <v>3.29</v>
-      </c>
+      <c r="B165" t="inlineStr"/>
+      <c r="C165" t="inlineStr"/>
+      <c r="D165" t="inlineStr"/>
+      <c r="E165" t="inlineStr"/>
       <c r="F165" t="n">
         <v>2352400</v>
       </c>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-01 23:57 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F165"/>
+  <dimension ref="A1:F167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3711,12 +3711,60 @@
       <c r="A165" s="1" t="n">
         <v>46262</v>
       </c>
-      <c r="B165" t="inlineStr"/>
-      <c r="C165" t="inlineStr"/>
-      <c r="D165" t="inlineStr"/>
-      <c r="E165" t="inlineStr"/>
+      <c r="B165" t="n">
+        <v>3.349999904632568</v>
+      </c>
+      <c r="C165" t="n">
+        <v>3.349999904632568</v>
+      </c>
+      <c r="D165" t="n">
+        <v>3.269999980926514</v>
+      </c>
+      <c r="E165" t="n">
+        <v>3.289999961853027</v>
+      </c>
       <c r="F165" t="n">
-        <v>2352400</v>
+        <v>2352700</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B166" t="n">
+        <v>3.440000057220459</v>
+      </c>
+      <c r="C166" t="n">
+        <v>3.450000047683716</v>
+      </c>
+      <c r="D166" t="n">
+        <v>3.339999914169312</v>
+      </c>
+      <c r="E166" t="n">
+        <v>3.359999895095825</v>
+      </c>
+      <c r="F166" t="n">
+        <v>5716600</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B167" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="C167" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="D167" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="E167" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="F167" t="n">
+        <v>4792100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-02 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F167"/>
+  <dimension ref="A1:F168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3752,19 +3752,39 @@
         <v>46266</v>
       </c>
       <c r="B167" t="n">
-        <v>3.56</v>
+        <v>3.559999942779541</v>
       </c>
       <c r="C167" t="n">
-        <v>3.6</v>
+        <v>3.599999904632568</v>
       </c>
       <c r="D167" t="n">
-        <v>3.42</v>
+        <v>3.420000076293945</v>
       </c>
       <c r="E167" t="n">
-        <v>3.43</v>
+        <v>3.430000066757202</v>
       </c>
       <c r="F167" t="n">
         <v>4792100</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="1" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B168" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="C168" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="D168" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="E168" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="F168" t="n">
+        <v>9978400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-03 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F168"/>
+  <dimension ref="A1:F169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3772,19 +3772,39 @@
         <v>46267</v>
       </c>
       <c r="B168" t="n">
-        <v>3.95</v>
+        <v>3.950000047683716</v>
       </c>
       <c r="C168" t="n">
-        <v>3.99</v>
+        <v>3.990000009536743</v>
       </c>
       <c r="D168" t="n">
-        <v>3.56</v>
+        <v>3.559999942779541</v>
       </c>
       <c r="E168" t="n">
-        <v>3.56</v>
+        <v>3.559999942779541</v>
       </c>
       <c r="F168" t="n">
         <v>9978400</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="1" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B169" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="C169" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="D169" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="E169" t="n">
+        <v>4</v>
+      </c>
+      <c r="F169" t="n">
+        <v>8161400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-04 22:26 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F169"/>
+  <dimension ref="A1:F170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3792,19 +3792,39 @@
         <v>46268</v>
       </c>
       <c r="B169" t="n">
-        <v>3.93</v>
+        <v>3.930000066757202</v>
       </c>
       <c r="C169" t="n">
-        <v>4.1</v>
+        <v>4.099999904632568</v>
       </c>
       <c r="D169" t="n">
-        <v>3.89</v>
+        <v>3.890000104904175</v>
       </c>
       <c r="E169" t="n">
         <v>4</v>
       </c>
       <c r="F169" t="n">
         <v>8161400</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="1" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B170" t="n">
+        <v>4</v>
+      </c>
+      <c r="C170" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="D170" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="E170" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F170" t="n">
+        <v>4564300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-07 22:26 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -3815,13 +3815,13 @@
         <v>4</v>
       </c>
       <c r="C170" t="n">
-        <v>4.05</v>
+        <v>4.050000190734863</v>
       </c>
       <c r="D170" t="n">
-        <v>3.9</v>
+        <v>3.900000095367432</v>
       </c>
       <c r="E170" t="n">
-        <v>3.9</v>
+        <v>3.900000095367432</v>
       </c>
       <c r="F170" t="n">
         <v>4564300</v>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-08 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F170"/>
+  <dimension ref="A1:F171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3827,6 +3827,26 @@
         <v>4564300</v>
       </c>
     </row>
+    <row r="171">
+      <c r="A171" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B171" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="C171" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="D171" t="n">
+        <v>4</v>
+      </c>
+      <c r="E171" t="n">
+        <v>4</v>
+      </c>
+      <c r="F171" t="n">
+        <v>5560900</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-09 22:28 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F171"/>
+  <dimension ref="A1:F172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3832,10 +3832,10 @@
         <v>46273</v>
       </c>
       <c r="B171" t="n">
-        <v>4.06</v>
+        <v>4.059999942779541</v>
       </c>
       <c r="C171" t="n">
-        <v>4.12</v>
+        <v>4.119999885559082</v>
       </c>
       <c r="D171" t="n">
         <v>4</v>
@@ -3845,6 +3845,26 @@
       </c>
       <c r="F171" t="n">
         <v>5560900</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B172" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="C172" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="D172" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="E172" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="F172" t="n">
+        <v>4528400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-10 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F172"/>
+  <dimension ref="A1:F173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3852,19 +3852,39 @@
         <v>46274</v>
       </c>
       <c r="B172" t="n">
-        <v>3.85</v>
+        <v>3.849999904632568</v>
       </c>
       <c r="C172" t="n">
-        <v>4.06</v>
+        <v>4.059999942779541</v>
       </c>
       <c r="D172" t="n">
-        <v>3.79</v>
+        <v>3.789999961853027</v>
       </c>
       <c r="E172" t="n">
-        <v>4.05</v>
+        <v>4.050000190734863</v>
       </c>
       <c r="F172" t="n">
         <v>4528400</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B173" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="C173" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="D173" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="E173" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="F173" t="n">
+        <v>4506600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MIA: run automatico 2026-09-11 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/AUAU3.xlsx
+++ b/database/AUAU3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F173"/>
+  <dimension ref="A1:F174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3872,19 +3872,39 @@
         <v>46275</v>
       </c>
       <c r="B173" t="n">
-        <v>4.03</v>
+        <v>4.03000020980835</v>
       </c>
       <c r="C173" t="n">
-        <v>4.03</v>
+        <v>4.03000020980835</v>
       </c>
       <c r="D173" t="n">
-        <v>3.8</v>
+        <v>3.799999952316284</v>
       </c>
       <c r="E173" t="n">
-        <v>3.81</v>
+        <v>3.809999942779541</v>
       </c>
       <c r="F173" t="n">
         <v>4506600</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="1" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B174" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="C174" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="D174" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="E174" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="F174" t="n">
+        <v>4859300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>